<commit_message>
Add 様/くん honorifics; decorate ballots with cat + hearts
- Roster: 名前 column now includes 「様」 (「くん」 for 守屋 陽杜)
- Ballots: rounded soft-blue cards, cat icon top-left, heart top-right,
  decorative dot line at bottom; dashed outer cutting line preserved

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015bCXw1XwjsCQKe2rGxWTfb
</commit_message>
<xml_diff>
--- a/attendees_roster.xlsx
+++ b/attendees_roster.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="出席者名簿" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="出席者名簿" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -469,7 +469,7 @@
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
@@ -522,7 +522,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>河合 直樹</t>
+          <t>河合 直樹 様</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -544,7 +544,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>加登 楓也</t>
+          <t>加登 楓也 様</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -566,7 +566,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>イ ギョム</t>
+          <t>イ ギョム 様</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
@@ -588,7 +588,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>阿南 心香</t>
+          <t>阿南 心香 様</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -610,7 +610,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>岡本 典子</t>
+          <t>岡本 典子 様</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -632,7 +632,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>趙 顯秀</t>
+          <t>趙 顯秀 様</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
@@ -654,7 +654,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>山根 直樹</t>
+          <t>山根 直樹 様</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
@@ -676,7 +676,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>森本 菜奈絵</t>
+          <t>森本 菜奈絵 様</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
@@ -698,7 +698,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>遠藤 優佳</t>
+          <t>遠藤 優佳 様</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
@@ -720,7 +720,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>永澤 友梨</t>
+          <t>永澤 友梨 様</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
@@ -742,7 +742,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>渡邊 彩音</t>
+          <t>渡邊 彩音 様</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
@@ -764,7 +764,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>周 孝海</t>
+          <t>周 孝海 様</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
@@ -786,7 +786,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>周 秀海</t>
+          <t>周 秀海 様</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
@@ -808,7 +808,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>周 伶海</t>
+          <t>周 伶海 様</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
@@ -830,7 +830,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>鈴木 亜海</t>
+          <t>鈴木 亜海 様</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
@@ -852,7 +852,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>宋 智子</t>
+          <t>宋 智子 様</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
@@ -874,7 +874,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>島田 崇司</t>
+          <t>島田 崇司 様</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
@@ -896,7 +896,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>飛松 虎太朗</t>
+          <t>飛松 虎太朗 様</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
@@ -918,7 +918,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>渡邊 雅之</t>
+          <t>渡邊 雅之 様</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
@@ -940,7 +940,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>中山 瑠惟</t>
+          <t>中山 瑠惟 様</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
@@ -962,7 +962,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>吉田 賢史</t>
+          <t>吉田 賢史 様</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
@@ -984,7 +984,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>津田 昂輝</t>
+          <t>津田 昂輝 様</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>安永 俊樹</t>
+          <t>安永 俊樹 様</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>昭元 公輝</t>
+          <t>昭元 公輝 様</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>森 貴裕</t>
+          <t>森 貴裕 様</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>大泉 周平</t>
+          <t>大泉 周平 様</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>守屋 勇汰</t>
+          <t>守屋 勇汰 様</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>守屋 陽杜</t>
+          <t>守屋 陽杜 くん</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>守屋 晴香</t>
+          <t>守屋 晴香 様</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>溝渕 比奈子</t>
+          <t>溝渕 比奈子 様</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
@@ -1182,7 +1182,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>畑中 聖奈</t>
+          <t>畑中 聖奈 様</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr"/>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>上原 夏紀</t>
+          <t>上原 夏紀 様</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr"/>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>橋村 ちゆき</t>
+          <t>橋村 ちゆき 様</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr"/>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>森口 小春</t>
+          <t>森口 小春 様</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr"/>
@@ -1270,7 +1270,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>渕上 綾香</t>
+          <t>渕上 綾香 様</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr"/>
@@ -1292,7 +1292,7 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>岩井 玲香</t>
+          <t>岩井 玲香 様</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>田中 真梨愛</t>
+          <t>田中 真梨愛 様</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr"/>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>野津 佳音</t>
+          <t>野津 佳音 様</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr"/>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>城戸 唯</t>
+          <t>城戸 唯 様</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr"/>
@@ -1380,7 +1380,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>田中 肖</t>
+          <t>田中 肖 様</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr"/>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>越澤 緑咲</t>
+          <t>越澤 緑咲 様</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr"/>
@@ -1424,7 +1424,7 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>宋 育子</t>
+          <t>宋 育子 様</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>宋 明良</t>
+          <t>宋 明良 様</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr"/>
@@ -1468,7 +1468,7 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>焦 美栄</t>
+          <t>焦 美栄 様</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr"/>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>宋 奈美季</t>
+          <t>宋 奈美季 様</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr"/>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>宋 宏樹</t>
+          <t>宋 宏樹 様</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr"/>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>宋 良夫</t>
+          <t>宋 良夫 様</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr"/>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>佐藤 嘉剛</t>
+          <t>佐藤 嘉剛 様</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr"/>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>佐藤 領祐</t>
+          <t>佐藤 領祐 様</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr"/>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>辻林 みゆ希</t>
+          <t>辻林 みゆ希 様</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr"/>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>門岡 綾希子</t>
+          <t>門岡 綾希子 様</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr"/>
@@ -1644,7 +1644,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>佐藤 公美子</t>
+          <t>佐藤 公美子 様</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr"/>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>濱本 泰延</t>
+          <t>濱本 泰延 様</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr"/>
@@ -1688,7 +1688,7 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>濱本 俊宏</t>
+          <t>濱本 俊宏 様</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr"/>
@@ -1710,7 +1710,7 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>濱岡 知子</t>
+          <t>濱岡 知子 様</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr"/>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>藤原 小矢佳</t>
+          <t>藤原 小矢佳 様</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr"/>
@@ -1754,7 +1754,7 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>瀧井 万友美</t>
+          <t>瀧井 万友美 様</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr"/>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>濱岡 香里</t>
+          <t>濱岡 香里 様</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr"/>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>阿南 悠乃</t>
+          <t>阿南 悠乃 様</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr"/>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>阿南 実穂乃</t>
+          <t>阿南 実穂乃 様</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr"/>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>阿南 純子</t>
+          <t>阿南 純子 様</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr"/>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>阿南 由紀</t>
+          <t>阿南 由紀 様</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr"/>
@@ -1886,7 +1886,7 @@
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>阿南 雅哉</t>
+          <t>阿南 雅哉 様</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr"/>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>阿南 洋一</t>
+          <t>阿南 洋一 様</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Split roster (友人/親族), add dress ballots, cute label
Roster:
- Two sheets: 友人 (A,B,D,E,F, 36名) and 親族 (C,G,H,I,J, 28名)
- Print setup: fit-to-page, 1st row repeats as print title

Ballots (7 slides, 4x4 grid, 104 slips total):
- Cat set (52 slips, soft blue) for 猫写真当て
- Dress set (52 slips, soft pink) for カラードレス色当て
- ♡ 投票用紙 ♡ label in cute pop font at top of each slip

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015bCXw1XwjsCQKe2rGxWTfb
</commit_message>
<xml_diff>
--- a/attendees_roster.xlsx
+++ b/attendees_roster.xlsx
@@ -7,9 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="出席者名簿" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="友人" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="親族" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'友人'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'親族'!$1:$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -38,7 +42,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -48,6 +52,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004A90D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9884A"/>
       </patternFill>
     </fill>
   </fills>
@@ -77,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -98,6 +107,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -461,9 +473,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -754,17 +766,17 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>新郎従弟</t>
+          <t>新郎新婦友人</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>周 孝海 様</t>
+          <t>島田 崇司 様</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
@@ -776,17 +788,17 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>新郎従弟</t>
+          <t>新郎新婦友人</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>周 秀海 様</t>
+          <t>飛松 虎太朗 様</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
@@ -798,17 +810,17 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>新郎従妹</t>
+          <t>新郎新婦友人</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>周 伶海 様</t>
+          <t>渡邊 雅之 様</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
@@ -820,17 +832,17 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>新郎従姉</t>
+          <t>新郎新婦友人</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>鈴木 亜海 様</t>
+          <t>中山 瑠惟 様</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
@@ -842,17 +854,17 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>新郎叔母</t>
+          <t>新郎新婦友人</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>宋 智子 様</t>
+          <t>吉田 賢史 様</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
@@ -874,7 +886,7 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>島田 崇司 様</t>
+          <t>津田 昂輝 様</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
@@ -896,7 +908,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>飛松 虎太朗 様</t>
+          <t>安永 俊樹 様</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
@@ -918,7 +930,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>渡邊 雅之 様</t>
+          <t>昭元 公輝 様</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
@@ -930,7 +942,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -940,7 +952,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>中山 瑠惟 様</t>
+          <t>森 貴裕 様</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
@@ -952,7 +964,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -962,7 +974,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>吉田 賢史 様</t>
+          <t>大泉 周平 様</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
@@ -974,7 +986,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -984,7 +996,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>津田 昂輝 様</t>
+          <t>守屋 勇汰 様</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
@@ -996,17 +1008,17 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>新郎新婦友人</t>
+          <t>新郎新婦友人御子息</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>安永 俊樹 様</t>
+          <t>守屋 陽杜 くん</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
@@ -1018,7 +1030,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1028,7 +1040,7 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>昭元 公輝 様</t>
+          <t>守屋 晴香 様</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
@@ -1050,7 +1062,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>森 貴裕 様</t>
+          <t>溝渕 比奈子 様</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
@@ -1072,7 +1084,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>大泉 周平 様</t>
+          <t>畑中 聖奈 様</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
@@ -1094,7 +1106,7 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>守屋 勇汰 様</t>
+          <t>上原 夏紀 様</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
@@ -1111,12 +1123,12 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>新郎新婦友人御子息</t>
+          <t>新郎新婦友人</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>守屋 陽杜 くん</t>
+          <t>橋村 ちゆき 様</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
@@ -1128,7 +1140,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -1138,7 +1150,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>守屋 晴香 様</t>
+          <t>森口 小春 様</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
@@ -1150,7 +1162,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -1160,7 +1172,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>溝渕 比奈子 様</t>
+          <t>渕上 綾香 様</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
@@ -1172,7 +1184,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -1182,7 +1194,7 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>畑中 聖奈 様</t>
+          <t>岩井 玲香 様</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr"/>
@@ -1194,7 +1206,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -1204,7 +1216,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>上原 夏紀 様</t>
+          <t>田中 真梨愛 様</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr"/>
@@ -1216,7 +1228,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -1226,7 +1238,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>橋村 ちゆき 様</t>
+          <t>野津 佳音 様</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr"/>
@@ -1248,7 +1260,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>森口 小春 様</t>
+          <t>城戸 唯 様</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr"/>
@@ -1270,7 +1282,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>渕上 綾香 様</t>
+          <t>田中 肖 様</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr"/>
@@ -1292,670 +1304,755 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>岩井 玲香 様</t>
+          <t>越澤 緑咲 様</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>新郎新婦友人</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>田中 真梨愛 様</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>新郎新婦友人</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>野津 佳音 様</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr"/>
-      <c r="F39" s="2" t="inlineStr"/>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>36名</t>
+        </is>
+      </c>
+      <c r="E38" s="6">
+        <f>COUNTIF(E2:E37,"〇")</f>
+        <v/>
+      </c>
+      <c r="F38" s="6">
+        <f>COUNTIF(F2:F37,"〇")</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>新郎新婦友人</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>城戸 唯 様</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr"/>
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>記入方法:</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>新郎新婦友人</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>田中 肖 様</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr"/>
-      <c r="F41" s="2" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>新郎新婦友人</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>越澤 緑咲 様</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>出席欄・お車欄に「〇」を入力すると自動集計されます。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>テーブル</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>続柄</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>名前</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>出席</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>お車</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>新郎従弟</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>周 孝海 様</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>新郎従弟</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>周 秀海 様</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>新郎従妹</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>周 伶海 様</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>新郎従姉</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>鈴木 亜海 様</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>新郎叔母</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>宋 智子 様</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>新郎母</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>宋 育子 様</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr"/>
-      <c r="F43" s="2" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="C44" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>新郎父</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>宋 明良 様</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>新郎祖母</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>焦 美栄 様</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr"/>
-      <c r="F45" s="2" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="C46" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>新郎妹</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>宋 奈美季 様</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>新郎弟</t>
         </is>
       </c>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>宋 宏樹 様</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr"/>
-      <c r="F47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="C48" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>新郎祖父</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>宋 良夫 様</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>新郎従弟</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>佐藤 嘉剛 様</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr"/>
-      <c r="F49" s="2" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="C50" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>新郎従兄</t>
         </is>
       </c>
-      <c r="D50" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>佐藤 領祐 様</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>新郎従姉</t>
         </is>
       </c>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>辻林 みゆ希 様</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr"/>
-      <c r="F51" s="2" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="C52" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>新郎従姉</t>
         </is>
       </c>
-      <c r="D52" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>門岡 綾希子 様</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr"/>
-      <c r="F52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>新郎叔母</t>
         </is>
       </c>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>佐藤 公美子 様</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr"/>
-      <c r="F53" s="2" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="C54" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>新郎従兄</t>
         </is>
       </c>
-      <c r="D54" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>濱本 泰延 様</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr"/>
-      <c r="F54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="C55" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>新郎従兄</t>
         </is>
       </c>
-      <c r="D55" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>濱本 俊宏 様</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr"/>
-      <c r="F55" s="2" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>新郎伯母</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>濱岡 知子 様</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr"/>
-      <c r="F56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="n">
-        <v>56</v>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>新郎従兄</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>藤原 小矢佳 様</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr"/>
-      <c r="F57" s="2" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>新郎従妹</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>瀧井 万友美 様</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr"/>
-      <c r="F58" s="2" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>新郎従妹</t>
         </is>
       </c>
-      <c r="D59" s="3" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>濱岡 香里 様</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr"/>
-      <c r="F59" s="2" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="C60" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>新婦姉</t>
         </is>
       </c>
-      <c r="D60" s="3" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>阿南 悠乃 様</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr"/>
-      <c r="F60" s="2" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>新婦妹</t>
         </is>
       </c>
-      <c r="D61" s="3" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>阿南 実穂乃 様</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr"/>
-      <c r="F61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="C62" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>新婦祖母</t>
         </is>
       </c>
-      <c r="D62" s="3" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>阿南 純子 様</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr"/>
-      <c r="F62" s="2" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="C63" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>新婦母</t>
         </is>
       </c>
-      <c r="D63" s="3" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>阿南 由紀 様</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr"/>
-      <c r="F63" s="2" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>新婦父</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>阿南 雅哉 様</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr"/>
-      <c r="F64" s="2" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="C65" s="3" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>新婦祖父</t>
         </is>
       </c>
-      <c r="D65" s="3" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>阿南 洋一 様</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr"/>
-      <c r="F65" s="2" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="C66" s="4" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t>64名</t>
-        </is>
-      </c>
-      <c r="E66" s="6">
-        <f>COUNTIF(E2:E65,"〇")</f>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>28名</t>
+        </is>
+      </c>
+      <c r="E30" s="6">
+        <f>COUNTIF(E2:E29,"〇")</f>
         <v/>
       </c>
-      <c r="F66" s="6">
-        <f>COUNTIF(F2:F65,"〇")</f>
+      <c r="F30" s="6">
+        <f>COUNTIF(F2:F29,"〇")</f>
         <v/>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="7" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>記入方法:</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>出席欄・お車欄に「〇」を入力すると自動集計されます。</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>例: 出席=〇 / 欠席=空欄, お車=〇（車で来場）/ 空欄（それ以外）</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix 濱本→濱岡 (Table I) in roster and ballots
User-corrected versions: 濱岡 泰延 様 and 濱岡 俊宏 様 in Table I
had been mistakenly extracted as 濱本 from the seating chart.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015bCXw1XwjsCQKe2rGxWTfb
</commit_message>
<xml_diff>
--- a/attendees_roster.xlsx
+++ b/attendees_roster.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yso13036.OFFICE\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4D75407-A4BE-4158-BFAC-555E80836CB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3125C454-EE50-4395-AEC6-B5E01CF5B40D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="312" yWindow="384" windowWidth="15120" windowHeight="12084" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="友人" sheetId="1" r:id="rId1"/>
@@ -292,12 +292,6 @@
     <t>I</t>
   </si>
   <si>
-    <t>濱本 泰延 様</t>
-  </si>
-  <si>
-    <t>濱本 俊宏 様</t>
-  </si>
-  <si>
     <t>新郎伯母</t>
   </si>
   <si>
@@ -361,6 +355,12 @@
   <si>
     <t>□</t>
     <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>濱岡 泰延 様</t>
+  </si>
+  <si>
+    <t>濱岡 俊宏 様</t>
   </si>
 </sst>
 </file>
@@ -832,7 +832,7 @@
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.4">
@@ -850,7 +850,7 @@
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.4">
@@ -884,7 +884,7 @@
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.4">
@@ -902,7 +902,7 @@
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.4">
@@ -968,7 +968,7 @@
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.4">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.4">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.4">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.4">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.4">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.4">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.4">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="E26" s="3"/>
       <c r="F26" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.4">
@@ -1449,7 +1449,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1734,11 +1734,11 @@
         <v>78</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>84</v>
+        <v>104</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.4">
@@ -1752,7 +1752,7 @@
         <v>78</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
@@ -1765,10 +1765,10 @@
         <v>83</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
@@ -1784,7 +1784,7 @@
         <v>78</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
@@ -1800,7 +1800,7 @@
         <v>57</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
@@ -1816,11 +1816,11 @@
         <v>57</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E23" s="3"/>
       <c r="F23" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.4">
@@ -1828,13 +1828,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D24" s="4" t="s">
         <v>91</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>93</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
@@ -1844,13 +1844,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
@@ -1860,13 +1860,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
@@ -1876,13 +1876,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
@@ -1892,13 +1892,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
@@ -1908,13 +1908,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>

</xml_diff>